<commit_message>
fix: product details nav
</commit_message>
<xml_diff>
--- a/backend/data/new_reviews.xlsx
+++ b/backend/data/new_reviews.xlsx
@@ -413,10 +413,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A2:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
@@ -536,6 +535,36 @@
       <c r="F5" t="inlineStr">
         <is>
           <t>2026-04-07 15:19:41.173000</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>69d755ef743954f368d29460</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>69d51bcba1be251df31ecd27</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>The product seems good and i am happy with it</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>69abed525a3b01606d0363f1</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-04-09 07:31:59.793059</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: cart removal #1
</commit_message>
<xml_diff>
--- a/backend/data/new_reviews.xlsx
+++ b/backend/data/new_reviews.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:F6"/>
+  <dimension ref="A2:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -565,6 +565,36 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>2026-04-09 07:31:59.793059</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>69ff43427a7c24c4d299bff7</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>69a5be2ce316a1020a47284a</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>the order arrived late and the packaging was awful</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>69fc2682e2f6b14a544e3557</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-05-09 14:22:58.364223</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: product ranking logic
</commit_message>
<xml_diff>
--- a/backend/data/new_reviews.xlsx
+++ b/backend/data/new_reviews.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:F7"/>
+  <dimension ref="A2:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -598,6 +598,96 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>69ff634953656ba68dffea2f</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>69ff5db68fe5b91c74c0a0a5</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Not satisfied with this product</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>69abe73d0fc72493a6e48704</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-05-09 16:39:37.321543</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>69ff74bac70c7ece4974d49f</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>69ff5db68fe5b91c74c0a0a5</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>The product seems good and i am happy with it</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>69fc22dbe2f6b14a544e3552</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-05-09 17:54:02.794905</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>69ff7517c70c7ece4974d4a1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>699ee05dee55d146d52ecd35</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>bad after sale service</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>69fc25efe2f6b14a544e3555</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-05-09 17:55:35.655743</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: "review collection and wilson score filter"
</commit_message>
<xml_diff>
--- a/backend/data/new_reviews.xlsx
+++ b/backend/data/new_reviews.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:F10"/>
+  <dimension ref="A2:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -554,7 +554,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>The product seems good and i am happy with it</t>
+          <t>The product seems good and i am happy with it.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -584,7 +584,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>the order arrived late and the packaging was awful</t>
+          <t>the order arrived late and the packaging was awful.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>bad after sale service</t>
+          <t>bad after sale service.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -685,6 +685,1056 @@
       <c r="F10" t="inlineStr">
         <is>
           <t>2026-05-09 17:55:35.655743</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>6a00245c2375c5b95b7733be</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>69ff5db68fe5b91c74c0a0a5</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>5</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Absolutely beast of a GPU, handles everything I throw at it</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>69ff79e7bd954abe2c592883</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-04-12 08:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>6a00245c2375c5b95b7733bf</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>69ff5db68fe5b91c74c0a0a5</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Blazing fast read speeds, huge upgrade from my old drive</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>69ff79e7bd954abe2c592890</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-04-12 08:10:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>6a00245c2375c5b95b7733c0</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>69ff5db68fe5b91c74c0a0a5</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Very quiet and keeps my CPU cool even under load</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>69ff79e7bd954abe2c592888</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-04-20 09:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>6a00245c2375c5b95b7733c1</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>69ff5db68fe5b91c74c0a0a5</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Great cable management, looks amazing with the glass panels</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>69ff79e7bd954abe2c592894</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-04-20 09:15:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>6a00245c2375c5b95b7733c2</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>6a001cba919268091de553eb</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Solid board, easy BIOS and stable with DDR5 at rated speeds</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>69ff79e7bd954abe2c592884</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-04-14 10:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>6a00245c2375c5b95b7733c3</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>6a001cba919268091de553eb</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>4</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>The LCD display on the pump head is a nice touch, cools well</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>69ff79e7bd954abe2c592889</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-04-14 10:20:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>6a00245c2375c5b95b7733c4</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>6a001cba919268091de553eb</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>5</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Colors are stunning, blacks are deep and response time is insane</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>69ff7f6ebd954abe2c5928c2</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-04-27 11:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>6a00245c2375c5b95b7733c5</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>6a001e0a919268091de553ed</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>5</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Excellent GPU, FSR 3 works really well for 4K gaming</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>69ff7f6ebd954abe2c5928b6</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-04-22 12:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>6a00245c2375c5b95b7733c6</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>6a001e0a919268091de553ed</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>5</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>PCIe 5.0 speeds are no joke, highly recommend for future builds</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>69ff7f6ebd954abe2c5928c9</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026-04-22 12:20:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>6a00245c2375c5b95b7733c7</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>6a001e0a919268091de553ed</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Does its job well, compatible with AM5 out of the box</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>69ff79e7bd954abe2c59288a</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>6a00245c2375c5b95b7733c8</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>6a001e0a919268091de553ed</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Great value mid-range board, no issues setting up Ryzen 7000</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>69ff79e7bd954abe2c592885</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:30:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>6a00245c2375c5b95b7733c9</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>6a001e32919268091de553ee</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>5</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>4K at 144Hz is a game changer, the curve feels natural</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>69ff7f6ebd954abe2c5928c3</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>6a00245c2375c5b95b7733ca</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>6a001e32919268091de553ee</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>4</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Fast and reliable, great for storing my whole game library</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>69ff7f6ebd954abe2c5928c7</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026-04-17 14:20:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>6a00245c2375c5b95b7733cb</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>6a001e32919268091de553ee</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>5</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Beautiful case, the triple glass view makes the build look premium</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>69ff7f6ebd954abe2c5928cc</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-05-04 09:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>6a00245c2375c5b95b7733cc</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>6a001e32919268091de553ee</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Top tier board, Thunderbolt 4 and 10GbE are very useful</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>69ff7f6ebd954abe2c5928bc</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-05-04 09:30:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>6a0028212375c5b95b7733d1</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>6a002788e8ae080766a97c86</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>5</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>The RTX 4090 is an absolute powerhouse,runs every game at max settings without breaking a sweat.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>69ff79e7bd954abe2c592883</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-04-22 10:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>6a0028212375c5b95b7733d2</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>6a002788e8ae080766a97c86USER_ID_ANIL</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Stopped working after two weeks, complete waste of money and the support team was useless.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>69ff7f6ebd954abe2c5928b6</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>2026-04-25 11:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>6a0028212375c5b95b7733d3</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>6a002788e8ae080766a97c86USER_ID_ANIL</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>decent motherboard, nothing special but works fine for a mid range build</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>69ff79e7bd954abe2c592884</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>2026-04-28 09:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>6a0028212375c5b95b7733d4</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>6a00279ee8ae080766a97c87</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>5</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>The OLED display is breathtaking, colors pop and the blacks are perfectly deep</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>69ff7f6ebd954abe2c5928c2</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2026-04-30 08:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>6a0028212375c5b95b7733d5</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>6a00279ee8ae080766a97c87</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>The drive failed after one month and I lost all my data, absolutely terrible product</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>69ff79e7bd954abe2c592890</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2026-05-01 10:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>6a0028212375c5b95b7733d6</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>6a00279ee8ae080766a97c87</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>5</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Keeps temperatures low and runs silently, very happy with this cooler</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>69ff79e7bd954abe2c592888</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-05-02 12:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>6a0028212375c5b95b7733d7</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>6a00279ee8ae080766a97c87</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Arrived damaged and the seller refused to replace it, very poor experience</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>69ff7f6ebd954abe2c5928c9</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>2026-05-03 09:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>6a0028212375c5b95b7733d8</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>6a0027b1e8ae080766a97c88</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>5</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>premium board with excellent build quality, the Thunderbolt 4 port is extremely useful</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>69ff7f6ebd954abe2c5928bc</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>2026-05-01 07:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>6a0028212375c5b95b7733d9</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>6a0027b1e8ae080766a97c88</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>the pump makes a loud rattling noise and the LCD display stopped working after a week</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>69ff79e7bd954abe2c592889</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2026-05-02 08:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>6a0028212375c5b95b7733da</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>6a0027b1e8ae080766a97c88</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>3</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Good monitor overall but the backlight bleeding is noticeable in dark scenes</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>69ff7f6ebd954abe2c5928c3</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-05-03 11:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>6a0028212375c5b95b7733db</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>6a0027b1e8ae080766a97c88</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Worst case I have ever owned, the glass panel cracked during installation and the screws stripped</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>69ff7f6ebd954abe2c5928cc</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>2026-05-04 10:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>6a0028212375c5b95b7733dc</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>6a0027c8e8ae080766a97c89</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>5</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>very stable with Ryzen 7000, BIOS updates were simple and DDR5 worked at full speed immediately</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>69ff79e7bd954abe2c592885</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2026-05-02 09:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>6a0028212375c5b95b7733dd</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>6a0027c8e8ae080766a97c89</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Average speed for the price, nothing impressive but gets the job done</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>69ff7f6ebd954abe2c5928c7</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>2026-05-03 10:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>6a0028212375c5b95b7733de</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>6a0027c8e8ae080766a97c89</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>2</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>not worth the price, runs hotter than expected and the fan is quite loud under load</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>69ff79e7bd954abe2c59288a</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>2026-05-04 08:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>6a0028212375c5b95b7733df</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>6a0027c8e8ae080766a97c89</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Cable management is a nightmare in this case, barely enough room behind the motherboard tray</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>69ff79e7bd954abe2c592894</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>2026-05-05 11:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>6a0028212375c5b95b7733e0</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>6a0027d9e8ae080766a97c8a</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Incredibly powerful GPU but runs extremely hot even with good airflow, thermal throttles under sustained load</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>69ff79e7bd954abe2c592883</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2026-05-03 07:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>6a0028212375c5b95b7733e1</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>6a0027d9e8ae080766a97c8a</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>burn in appeared after just three months of normal use, extremely disappointed for this price</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>69ff7f6ebd954abe2c5928c2</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>2026-05-04 09:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>6a0028212375c5b95b7733e2</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>6a0027d9e8ae080766a97c8a</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>4</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Solid GPU for 4K gaming, FSR 3 works great and the card stays cool and quiet</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>69ff7f6ebd954abe2c5928b6</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>2026-05-05 10:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>6a0028212375c5b95b7733e3</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>6a0027d9e8ae080766a97c8a</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>5</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Incredibly fast SSD, boot times are under ten seconds and large file transfers finish almost instantly</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>69ff79e7bd954abe2c592890</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>2026-05-06 08:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>6a004437166836f13eb6f9b9</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>6a0027c8e8ae080766a97c89</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Stopped working after two weeks, complete waste of money and the support team was useless.</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>69ff79e7bd954abe2c59288c</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2026-05-10 08:39:19.523116</t>
         </is>
       </c>
     </row>

</xml_diff>